<commit_message>
From GFG Greatest of three numbers problem solved
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -563,10 +563,16 @@
       <c r="A12" t="s">
         <v>11</v>
       </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
From hackerrank Max Min problem solved
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -579,10 +579,16 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
+      <c r="B14" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
From GFG Sum of Digits problem solved
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -596,82 +596,88 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
Factorial of a number done
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>Logic done</t>
+  </si>
+  <si>
+    <t>Logic Done</t>
   </si>
 </sst>
 </file>
@@ -595,6 +598,9 @@
       <c r="A16" t="s">
         <v>15</v>
       </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -604,6 +610,9 @@
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
From HackerEarth Calculate the Power code done
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -622,6 +622,9 @@
       <c r="A19" t="s">
         <v>18</v>
       </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">

</xml_diff>

<commit_message>
From GFG Number of factors problem solved
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="38">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -630,6 +630,9 @@
       <c r="A20" t="s">
         <v>19</v>
       </c>
+      <c r="B20" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">

</xml_diff>

<commit_message>
From GFG STRONG NUMBER problem solved
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="38">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -643,6 +643,9 @@
       <c r="A22" t="s">
         <v>21</v>
       </c>
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">

</xml_diff>

<commit_message>
Check if a Number is Automorphic problem solved
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -651,6 +651,9 @@
       <c r="A23" t="s">
         <v>22</v>
       </c>
+      <c r="B23" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">

</xml_diff>

<commit_message>
LCM of two numbers SOLVED
</commit_message>
<xml_diff>
--- a/NUMBERS_AND_MATH.xlsx
+++ b/NUMBERS_AND_MATH.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="38">
   <si>
     <t>Check if a number is palindrome or not</t>
   </si>
@@ -667,6 +667,9 @@
       <c r="A25" t="s">
         <v>24</v>
       </c>
+      <c r="B25" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">

</xml_diff>